<commit_message>
Medate fiels req field
</commit_message>
<xml_diff>
--- a/TestData/LV_T1693_ValidationsToBeCompletedBeforeFROpportunityIsApproved.xlsx
+++ b/TestData/LV_T1693_ValidationsToBeCompletedBeforeFROpportunityIsApproved.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A903E907-AE3F-4B1C-8672-4024EFD20B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F185C44-A3C2-4841-8DD0-C48B96C283E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -335,7 +335,7 @@
     <t>BUS - Business Services</t>
   </si>
   <si>
-    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Marketing--&gt;Information: Client Description is required.Marketing--&gt;Information: Select \"Total Debt(MM) Confirmed\" checkbox to confirm Total Debt is most up to date.Marketing--&gt;Information: Total Debt HL represents(MM), input zero if not applicable.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Client/Subject &amp; Referral--&gt;Referral Info: Referral Type is required.Client/Subject &amp; Referral--&gt;Referral Info: Legal Advisor to Company is required.Client/Subject &amp; Referral--&gt;Referral Info: Legal Advisor to HL Client Group is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Location where Service Benefit was provided is required.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
+    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Marketing--&gt;Information: Client Description is required.Marketing--&gt;Information: Select \"Total Debt(MM) Confirmed\" checkbox to confirm Total Debt is most up to date.Marketing--&gt;Information: Total Debt HL represents(MM), input zero if not applicable.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Client/Subject &amp; Referral--&gt;Referral Info: Referral Type is required.Client/Subject &amp; Referral--&gt;Referral Info: Legal Advisor to Company is required.Client/Subject &amp; Referral--&gt;Referral Info: Legal Advisor to HL Client Group is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Location where Service Benefit was provided is required.Info--&gt;Administration: Estimated Close Date is required.Pitches/Mandate Awards: A Pitch/Mandate's Outcome is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
   </si>
 </sst>
 </file>

</xml_diff>